<commit_message>
Retire CBS CSV service and refresh packaged metadata
- Remove the retired CBS CSV SFTP account: no automatic fallback, explicit
  legacy connections are rejected, and its 154 catalog rows are dropped.
  CSV readers, processing and output are unchanged.
- Add Ownership History links_2025 (CBS SFTP export confirmed 2026-10-29)
  to the catalog, both dictionaries, date metadata and batch template, and
  point the product at its new top-level directory Xd0wpsp9TCSp6AdYQYSBTQ.
- Restore provider Type/Remarks from Orbis Data Dictionary v1, backfill
  targeted remarks, and repair UTF-8 mojibake in imported text.
- Track dataset availability in ROADMAP.md and TODO.md.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/moodys_datahub/data/date_cols.xlsx
+++ b/src/moodys_datahub/data/date_cols.xlsx
@@ -17,7 +17,7 @@
     <sheet name="Ark1" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$D$131</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$D$132</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -928,7 +928,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D131"/>
+  <dimension ref="A1:D132"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="55.5703125" style="1" customWidth="1"/>
@@ -1291,8 +1291,10 @@
       <c r="A26" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="B26" s="1" t="s">
-        <v>169</v>
+      <c r="B26" s="1" t="inlineStr">
+        <is>
+          <t>status_history, statushistory</t>
+        </is>
       </c>
       <c r="C26" s="1" t="s">
         <v>119</v>
@@ -2771,10 +2773,26 @@
         <v>158</v>
       </c>
     </row>
+    <row r="132" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A132" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B132" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">links_2025</t>
+        </is>
+      </c>
+      <c r="C132" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D132" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D131" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D129">
-      <sortCondition ref="A1:A129"/>
+  <autoFilter ref="A1:D132" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D132">
+      <sortCondition ref="A1:A132"/>
     </sortState>
   </autoFilter>
   <phoneticPr fontId="3" type="noConversion"/>

</xml_diff>